<commit_message>
fix: remove crypto from proxy, use AUTH_SECRET directly as session token
</commit_message>
<xml_diff>
--- a/자산관리_업로드양식_260618.xlsx
+++ b/자산관리_업로드양식_260618.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
   <si>
     <t>자산구분</t>
   </si>
@@ -98,124 +98,150 @@
     <t>005930</t>
   </si>
   <si>
+    <t>주식</t>
+  </si>
+  <si>
+    <t>069500</t>
+  </si>
+  <si>
+    <t>거래일자</t>
+  </si>
+  <si>
+    <t>거래구분</t>
+  </si>
+  <si>
+    <t>거래수량</t>
+  </si>
+  <si>
+    <t>거래단가(원)</t>
+  </si>
+  <si>
+    <t>거래금액(원)</t>
+  </si>
+  <si>
+    <t>수수료(원)</t>
+  </si>
+  <si>
+    <t>세금(원)</t>
+  </si>
+  <si>
+    <t>순손익(원)</t>
+  </si>
+  <si>
+    <t>2025-01-15</t>
+  </si>
+  <si>
+    <t>매수</t>
+  </si>
+  <si>
+    <t>2025-03-20</t>
+  </si>
+  <si>
+    <t>은행</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IM뱅크</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>저축예금</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KDB생명</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1234-56-7891</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>삼천리</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>삼성전자</t>
-  </si>
-  <si>
-    <t>주식</t>
-  </si>
-  <si>
-    <t>069500</t>
-  </si>
-  <si>
-    <t>거래일자</t>
-  </si>
-  <si>
-    <t>거래구분</t>
-  </si>
-  <si>
-    <t>거래수량</t>
-  </si>
-  <si>
-    <t>거래단가(원)</t>
-  </si>
-  <si>
-    <t>거래금액(원)</t>
-  </si>
-  <si>
-    <t>수수료(원)</t>
-  </si>
-  <si>
-    <t>세금(원)</t>
-  </si>
-  <si>
-    <t>순손익(원)</t>
-  </si>
-  <si>
-    <t>2025-01-15</t>
-  </si>
-  <si>
-    <t>매수</t>
-  </si>
-  <si>
-    <t>2025-03-20</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAVER</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>JYP Ent.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TIGER 미국배당다우존스</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODEX 미국배당커버드콜액티브</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODEX 미국AI전력핵심인프라</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>하이브</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>오스테오닉</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>플라즈맵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODEX 고배당주</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TIGER 미국배당다우존스</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TIGER 미국배당다우존스타겟커버드콜1호</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ETF</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IRP</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODEX 차이나기술</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KODEX 채권</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ACE 반도체ETF</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>현대차</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>미래에셋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>매도</t>
-  </si>
-  <si>
-    <t>은행</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>IM뱅크</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>저축예금</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KDB생명</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>1234-56-7891</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>삼천리</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>삼성전자</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>NAVER</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>JYP Ent.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>TIGER 미국배당다우존스</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KODEX 미국배당커버드콜액티브</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KODEX 미국AI전력핵심인프라</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>하이브</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>오스테오닉</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>플라즈맵</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KODEX 고배당주</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>TIGER 미국배당다우존스</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>TIGER 미국배당다우존스타겟커버드콜1호</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ETF</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>메도</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -283,11 +309,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="백분율" xfId="1" builtinId="5"/>
@@ -671,7 +698,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -688,16 +715,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>42</v>
-      </c>
-      <c r="D3" t="s">
-        <v>44</v>
       </c>
       <c r="E3" s="1">
         <v>55153</v>
@@ -714,7 +741,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -747,11 +774,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.5546875" customWidth="1"/>
-    <col min="4" max="6" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.33203125" customWidth="1"/>
     <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -790,10 +818,10 @@
         <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D2" s="3">
         <v>42</v>
@@ -818,13 +846,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D3" s="3">
         <v>55</v>
@@ -839,20 +867,20 @@
         <v>19566250</v>
       </c>
       <c r="H3" s="3">
-        <f t="shared" ref="H3:H14" si="0">(F3-E3)*D3</f>
+        <f t="shared" ref="H3:H17" si="0">(F3-E3)*D3</f>
         <v>11503250</v>
       </c>
       <c r="I3" s="2">
-        <f t="shared" ref="I3:I14" si="1">H3/(E3*D3)</f>
+        <f t="shared" ref="I3:I17" si="1">H3/(E3*D3)</f>
         <v>1.4266712141882674</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" s="3">
         <v>20</v>
@@ -877,10 +905,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" s="3">
         <v>70</v>
@@ -905,10 +933,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3">
         <v>189</v>
@@ -933,10 +961,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D7" s="3">
         <v>2417</v>
@@ -961,10 +989,10 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D8" s="3">
         <v>169</v>
@@ -989,10 +1017,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D9" s="3">
         <v>13</v>
@@ -1017,10 +1045,10 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3">
         <v>1500</v>
@@ -1045,10 +1073,10 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D11" s="3">
         <v>536</v>
@@ -1073,10 +1101,10 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3">
         <v>500</v>
@@ -1101,10 +1129,10 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
         <v>56</v>
-      </c>
-      <c r="C13" t="s">
-        <v>58</v>
       </c>
       <c r="D13" s="3">
         <v>742</v>
@@ -1129,10 +1157,10 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D14" s="3">
         <v>866</v>
@@ -1153,6 +1181,93 @@
       <c r="I14" s="2">
         <f t="shared" si="1"/>
         <v>8.9401294498381884E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="3">
+        <v>100</v>
+      </c>
+      <c r="E15" s="3">
+        <v>230000</v>
+      </c>
+      <c r="F15" s="3">
+        <v>260000</v>
+      </c>
+      <c r="G15" s="3">
+        <f>D15*F15</f>
+        <v>26000000</v>
+      </c>
+      <c r="H15" s="3">
+        <f t="shared" si="0"/>
+        <v>3000000</v>
+      </c>
+      <c r="I15" s="2">
+        <f t="shared" si="1"/>
+        <v>0.13043478260869565</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="3">
+        <v>100</v>
+      </c>
+      <c r="E16" s="3">
+        <v>350000</v>
+      </c>
+      <c r="F16" s="3">
+        <v>365000</v>
+      </c>
+      <c r="G16" s="3">
+        <f t="shared" ref="G16:G17" si="2">D16*F16</f>
+        <v>36500000</v>
+      </c>
+      <c r="H16" s="3">
+        <f t="shared" si="0"/>
+        <v>1500000</v>
+      </c>
+      <c r="I16" s="2">
+        <f t="shared" si="1"/>
+        <v>4.2857142857142858E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="3">
+        <v>100</v>
+      </c>
+      <c r="E17" s="3">
+        <v>210000</v>
+      </c>
+      <c r="F17" s="3">
+        <v>450000</v>
+      </c>
+      <c r="G17" s="3">
+        <f t="shared" si="2"/>
+        <v>45000000</v>
+      </c>
+      <c r="H17" s="3">
+        <f t="shared" si="0"/>
+        <v>24000000</v>
+      </c>
+      <c r="I17" s="2">
+        <f t="shared" si="1"/>
+        <v>1.1428571428571428</v>
       </c>
     </row>
   </sheetData>
@@ -1167,12 +1282,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
         <v>15</v>
@@ -1181,96 +1302,144 @@
         <v>16</v>
       </c>
       <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>33</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>34</v>
-      </c>
-      <c r="J1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2">
+        <v>36</v>
+      </c>
+      <c r="E2" s="4">
         <v>50</v>
       </c>
-      <c r="F2">
-        <v>68000</v>
-      </c>
-      <c r="G2">
+      <c r="F2" s="4"/>
+      <c r="G2" s="4">
         <v>3400000</v>
       </c>
-      <c r="H2">
-        <v>5100</v>
-      </c>
-      <c r="I2">
+      <c r="H2" s="4">
+        <f>G2*0.1%</f>
+        <v>3400</v>
+      </c>
+      <c r="I2" s="4">
         <v>0</v>
       </c>
-      <c r="J2">
-        <v>-5100</v>
+      <c r="J2" s="4">
+        <f>-H2</f>
+        <v>-3400</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3">
-        <v>20</v>
-      </c>
-      <c r="F3">
-        <v>75000</v>
-      </c>
-      <c r="G3">
-        <v>1500000</v>
-      </c>
-      <c r="H3">
-        <v>2250</v>
-      </c>
-      <c r="I3">
-        <v>2250</v>
-      </c>
-      <c r="J3">
-        <v>135500</v>
+        <v>63</v>
+      </c>
+      <c r="E3" s="4">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4">
+        <v>7600000</v>
+      </c>
+      <c r="H3" s="4">
+        <f>G3*0.1%</f>
+        <v>7600</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <f>G3-G2-H3</f>
+        <v>4192400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4">
+        <v>2100000</v>
+      </c>
+      <c r="H4" s="4">
+        <f>G4*0.1%</f>
+        <v>2100</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <f>-H4</f>
+        <v>-2100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4">
+        <v>5600000</v>
+      </c>
+      <c r="H5" s="4">
+        <f>G5*0.1%</f>
+        <v>5600</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <f>G5-G4-H5</f>
+        <v>3494400</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 A2:B3 D2:E2 G2 I2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: TOP 20 stocks real-time data via Yahoo Finance API
</commit_message>
<xml_diff>
--- a/자산관리_업로드양식_260618.xlsx
+++ b/자산관리_업로드양식_260618.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="86">
   <si>
     <t>자산구분</t>
   </si>
@@ -242,6 +242,75 @@
   </si>
   <si>
     <t>메도</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>은행</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>농협은행</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>123-425-7853</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>069501</t>
+  </si>
+  <si>
+    <t>069502</t>
+  </si>
+  <si>
+    <t>069503</t>
+  </si>
+  <si>
+    <t>069504</t>
+  </si>
+  <si>
+    <t>069505</t>
+  </si>
+  <si>
+    <t>069506</t>
+  </si>
+  <si>
+    <t>069507</t>
+  </si>
+  <si>
+    <t>069508</t>
+  </si>
+  <si>
+    <t>069509</t>
+  </si>
+  <si>
+    <t>069510</t>
+  </si>
+  <si>
+    <t>069511</t>
+  </si>
+  <si>
+    <t>069512</t>
+  </si>
+  <si>
+    <t>069513</t>
+  </si>
+  <si>
+    <t>069514</t>
+  </si>
+  <si>
+    <t>`</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>069515</t>
+  </si>
+  <si>
+    <t>테슬라</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>주식</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -309,12 +378,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="백분율" xfId="1" builtinId="5"/>
@@ -656,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="32.44140625" customWidth="1"/>
@@ -738,27 +810,50 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="1">
+        <v>55153</v>
+      </c>
+      <c r="F4">
+        <v>6500000</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E5" s="1">
         <v>58498</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>83083517</v>
       </c>
-      <c r="G4">
+      <c r="G5">
         <v>3</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -767,14 +862,14 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A4 A1:H1 A2:B2 D2 C4:D4 H4" numberStoredAsText="1"/>
+    <ignoredError sqref="A5 A1:H1 A2:B2 D2 C5:D5 H5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.5546875" customWidth="1"/>
@@ -823,19 +918,19 @@
       <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="5">
         <v>42</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="5">
         <v>120100</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="5">
         <v>120500</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="5">
         <v>5061000</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="5">
         <f>(F2-E2)*D2</f>
         <v>16800</v>
       </c>
@@ -854,47 +949,50 @@
       <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="5">
         <v>55</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="5">
         <v>146600</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="5">
         <v>355750</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="5">
         <v>19566250</v>
       </c>
-      <c r="H3" s="3">
-        <f t="shared" ref="H3:H17" si="0">(F3-E3)*D3</f>
+      <c r="H3" s="5">
+        <f t="shared" ref="H3:H18" si="0">(F3-E3)*D3</f>
         <v>11503250</v>
       </c>
       <c r="I3" s="2">
-        <f t="shared" ref="I3:I17" si="1">H3/(E3*D3)</f>
+        <f t="shared" ref="I3:I18" si="1">H3/(E3*D3)</f>
         <v>1.4266712141882674</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>68</v>
+      </c>
       <c r="B4" t="s">
         <v>45</v>
       </c>
       <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="5">
         <v>20</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="5">
         <v>253000</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="5">
         <v>236500</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="5">
         <v>4730000</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="5">
         <f t="shared" si="0"/>
         <v>-330000</v>
       </c>
@@ -904,25 +1002,28 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>69</v>
+      </c>
       <c r="B5" t="s">
         <v>46</v>
       </c>
       <c r="C5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>70</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>69800</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="5">
         <v>55800</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="5">
         <v>3906000</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="5">
         <f t="shared" si="0"/>
         <v>-980000</v>
       </c>
@@ -932,25 +1033,28 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
       <c r="B6" t="s">
         <v>48</v>
       </c>
       <c r="C6" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="5">
         <v>189</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="5">
         <v>12277</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="5">
         <v>13520</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="5">
         <v>2555280</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="5">
         <f t="shared" si="0"/>
         <v>234927</v>
       </c>
@@ -960,25 +1064,28 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>71</v>
+      </c>
       <c r="B7" t="s">
         <v>47</v>
       </c>
       <c r="C7" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>2417</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="5">
         <v>13896</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="5">
         <v>15465</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="5">
         <v>37378905</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="5">
         <f t="shared" si="0"/>
         <v>3792273</v>
       </c>
@@ -988,25 +1095,28 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>72</v>
+      </c>
       <c r="B8" t="s">
         <v>49</v>
       </c>
       <c r="C8" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="5">
         <v>169</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>17886</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="5">
         <v>26569.8224852071</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="5">
         <v>4490300</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="5">
         <f t="shared" si="0"/>
         <v>1467565.9999999998</v>
       </c>
@@ -1016,25 +1126,28 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
       <c r="B9" t="s">
         <v>50</v>
       </c>
       <c r="C9" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="5">
         <v>13</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>302500</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="5">
         <v>226500</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="5">
         <v>2944500</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="5">
         <f t="shared" si="0"/>
         <v>-988000</v>
       </c>
@@ -1044,25 +1157,28 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
       <c r="B10" t="s">
         <v>51</v>
       </c>
       <c r="C10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="5">
         <v>1500</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="5">
         <v>5146</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="5">
         <v>4360</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="5">
         <v>6540000</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="5">
         <f t="shared" si="0"/>
         <v>-1179000</v>
       </c>
@@ -1072,25 +1188,28 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>75</v>
+      </c>
       <c r="B11" t="s">
         <v>52</v>
       </c>
       <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <v>536</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>13049</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="5">
         <v>3925</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="5">
         <v>2103800</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="5">
         <f t="shared" si="0"/>
         <v>-4890464</v>
       </c>
@@ -1100,25 +1219,28 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
       <c r="B12" t="s">
         <v>53</v>
       </c>
       <c r="C12" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="5">
         <v>500</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>14210</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="5">
         <v>17720</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="5">
         <v>8860000</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="5">
         <f t="shared" si="0"/>
         <v>1755000</v>
       </c>
@@ -1128,25 +1250,28 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
       <c r="B13" t="s">
         <v>54</v>
       </c>
       <c r="C13" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="5">
         <v>742</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="5">
         <v>14815</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="5">
         <v>15465</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="5">
         <v>11475030</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="5">
         <f t="shared" si="0"/>
         <v>482300</v>
       </c>
@@ -1156,25 +1281,28 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
       <c r="B14" t="s">
         <v>55</v>
       </c>
       <c r="C14" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="5">
         <v>866</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="5">
         <v>12360</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="5">
         <v>13465</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="5">
         <v>11660690</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="5">
         <f t="shared" si="0"/>
         <v>956930</v>
       </c>
@@ -1184,26 +1312,28 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>79</v>
+      </c>
       <c r="B15" t="s">
         <v>58</v>
       </c>
       <c r="C15" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="5">
         <v>100</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="5">
         <v>230000</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="5">
         <v>260000</v>
       </c>
-      <c r="G15" s="3">
-        <f>D15*F15</f>
+      <c r="G15" s="5">
         <v>26000000</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="5">
         <f t="shared" si="0"/>
         <v>3000000</v>
       </c>
@@ -1213,26 +1343,28 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>80</v>
+      </c>
       <c r="B16" t="s">
         <v>59</v>
       </c>
       <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="5">
         <v>100</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="5">
         <v>350000</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="5">
         <v>365000</v>
       </c>
-      <c r="G16" s="3">
-        <f t="shared" ref="G16:G17" si="2">D16*F16</f>
+      <c r="G16" s="5">
         <v>36500000</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="5">
         <f t="shared" si="0"/>
         <v>1500000</v>
       </c>
@@ -1241,33 +1373,66 @@
         <v>4.2857142857142858E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>81</v>
+      </c>
       <c r="B17" t="s">
         <v>60</v>
       </c>
       <c r="C17" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="5">
         <v>100</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="5">
         <v>210000</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="5">
         <v>450000</v>
       </c>
-      <c r="G17" s="3">
-        <f t="shared" si="2"/>
+      <c r="G17" s="5">
         <v>45000000</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="5">
         <f t="shared" si="0"/>
         <v>24000000</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" si="1"/>
         <v>1.1428571428571428</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="5">
+        <v>30</v>
+      </c>
+      <c r="E18" s="5">
+        <v>250000</v>
+      </c>
+      <c r="F18" s="5">
+        <v>620000</v>
+      </c>
+      <c r="G18" s="3">
+        <v>18600000</v>
+      </c>
+      <c r="H18" s="5">
+        <f t="shared" si="0"/>
+        <v>11100000</v>
+      </c>
+      <c r="I18" s="2">
+        <f t="shared" si="1"/>
+        <v>1.48</v>
       </c>
     </row>
   </sheetData>
@@ -1282,7 +1447,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
@@ -1291,7 +1456,7 @@
     <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1323,11 +1488,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>35</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C2" t="s">
@@ -1336,30 +1501,30 @@
       <c r="D2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>50</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3">
         <v>3400000</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="3">
         <f>G2*0.1%</f>
         <v>3400</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="3">
         <v>0</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="3">
         <f>-H2</f>
         <v>-3400</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>37</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C3" t="s">
@@ -1368,71 +1533,92 @@
       <c r="D3" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>50</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4">
+      <c r="F3" s="3"/>
+      <c r="G3" s="3">
         <v>7600000</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <f>G3*0.1%</f>
         <v>7600</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>0</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="3">
         <f>G3-G2-H3</f>
         <v>4192400</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="4">
+        <v>5933</v>
+      </c>
       <c r="C4" t="s">
         <v>62</v>
       </c>
       <c r="D4" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4">
+      <c r="E4" s="3">
+        <v>100</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3">
         <v>2100000</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <f>G4*0.1%</f>
         <v>2100</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>0</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <f>-H4</f>
         <v>-2100</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="4">
+        <v>5933</v>
+      </c>
       <c r="C5" t="s">
         <v>62</v>
       </c>
       <c r="D5" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4">
+      <c r="E5" s="3">
+        <v>100</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3">
         <v>5600000</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <f>G5*0.1%</f>
         <v>5600</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="3">
         <v>0</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="3">
         <f>G5-G4-H5</f>
         <v>3494400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L8" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>